<commit_message>
Add provincial sect societies, estates, trials, and diplomacy
</commit_message>
<xml_diff>
--- a/outputs/aura-clash-events/AuraClash-event-tracker.xlsx
+++ b/outputs/aura-clash-events/AuraClash-event-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" r:id="Rfe051484b2e345f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="R95b62c729e1543d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" r:id="Rd53deb5b7af845a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="Rf579f303f8b24cc2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -643,7 +643,7 @@
         <x:v>events/dlc/tgp/tgp_japan_yearly_events_ariana.txt:5213</x:v>
       </x:c>
       <x:c r="G11" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:3160</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:3159</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="36" customHeight="1">
@@ -804,7 +804,7 @@
         <x:v>events/dlc/tgp/tgp_governor_contract_events.txt:2872</x:v>
       </x:c>
       <x:c r="G18" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2326</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2325</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="32" customHeight="1">
@@ -873,7 +873,7 @@
         <x:v>events/dlc/tgp/tgp_natural_disaster_flavor_events.txt:585</x:v>
       </x:c>
       <x:c r="G21" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2497</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2496</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="36" customHeight="1">
@@ -965,7 +965,7 @@
         <x:v>events/dlc/tgp/tgp_natural_disaster_flavor_events.txt:259</x:v>
       </x:c>
       <x:c r="G25" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2836</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2835</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="36" customHeight="1">
@@ -1034,7 +1034,7 @@
         <x:v>events/travel_events/travel_danger_events_arky.txt:143</x:v>
       </x:c>
       <x:c r="G28" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4399</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4398</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="36" customHeight="1">
@@ -1057,7 +1057,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:529</x:v>
       </x:c>
       <x:c r="G29" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10960</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10959</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="36" customHeight="1">
@@ -1080,7 +1080,7 @@
         <x:v>events/health_events.txt:9507</x:v>
       </x:c>
       <x:c r="G30" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_health_options.txt:295</x:v>
+        <x:v>AuraClash/events/ac_vanilla_health_options.txt:294</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="36" customHeight="1">
@@ -1126,7 +1126,7 @@
         <x:v>events/activities/hunt_activity/hunt_events_anna.txt:437</x:v>
       </x:c>
       <x:c r="G32" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10137</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10136</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="36" customHeight="1">
@@ -1149,7 +1149,7 @@
         <x:v>events/activities/feast_activity/main_events/feast_default_events.txt:12335</x:v>
       </x:c>
       <x:c r="G33" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11810</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11809</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="36" customHeight="1">
@@ -1172,7 +1172,7 @@
         <x:v>events/travel_events/travel_events.txt:880</x:v>
       </x:c>
       <x:c r="G34" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4201</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4200</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="36" customHeight="1">
@@ -1195,7 +1195,7 @@
         <x:v>events/travel_events/travel_danger_events_joe.txt:135</x:v>
       </x:c>
       <x:c r="G35" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6015</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6014</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="36" customHeight="1">
@@ -1218,7 +1218,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:1466</x:v>
       </x:c>
       <x:c r="G36" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1318</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1317</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="36" customHeight="1">
@@ -1241,7 +1241,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:582</x:v>
       </x:c>
       <x:c r="G37" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1883</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1882</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="36" customHeight="1">
@@ -1264,7 +1264,7 @@
         <x:v>events/travel_events/travel_events_veronica.txt:3064</x:v>
       </x:c>
       <x:c r="G38" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3006</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3005</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="36" customHeight="1">
@@ -1287,7 +1287,7 @@
         <x:v>events/travel_events/travel_danger_events_joe.txt:2211</x:v>
       </x:c>
       <x:c r="G39" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_fatal_options.txt:17</x:v>
+        <x:v>AuraClash/events/ac_vanilla_fatal_options.txt:16</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="36" customHeight="1">
@@ -1310,7 +1310,7 @@
         <x:v>events/travel_events/travel_danger_events.txt:613</x:v>
       </x:c>
       <x:c r="G40" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:2214</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:2213</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="36" customHeight="1">
@@ -1333,7 +1333,7 @@
         <x:v>events/travel_events/travel_events_veronica.txt:4531</x:v>
       </x:c>
       <x:c r="G41" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:7107</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:7106</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="36" customHeight="1">
@@ -1356,7 +1356,7 @@
         <x:v>events/travel_events/travel_danger_events_joe.txt:2364</x:v>
       </x:c>
       <x:c r="G42" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3334</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3333</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="36" customHeight="1">
@@ -1379,7 +1379,7 @@
         <x:v>events/travel_events/travel_danger_events.txt:806</x:v>
       </x:c>
       <x:c r="G43" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1132</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1131</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="36" customHeight="1">
@@ -1402,7 +1402,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:9</x:v>
       </x:c>
       <x:c r="G44" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:2420</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:2419</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="36" customHeight="1">
@@ -1425,7 +1425,7 @@
         <x:v>events/travel_events/travel_danger_events_filippa.txt:8</x:v>
       </x:c>
       <x:c r="G45" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:608</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:607</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="36" customHeight="1">
@@ -1448,7 +1448,7 @@
         <x:v>events/travel_events/travel_danger_events_oltner.txt:922</x:v>
       </x:c>
       <x:c r="G46" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4039</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4038</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="36" customHeight="1">
@@ -1471,7 +1471,7 @@
         <x:v>events/travel_events/travel_danger_events_ariana.txt:92</x:v>
       </x:c>
       <x:c r="G47" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:5058</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:5057</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="36" customHeight="1">
@@ -1494,7 +1494,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:949</x:v>
       </x:c>
       <x:c r="G48" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1544</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1543</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="36" customHeight="1">
@@ -1517,7 +1517,7 @@
         <x:v>events/travel_events/travel_danger_events_oltner.txt:301</x:v>
       </x:c>
       <x:c r="G49" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:3005</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:3004</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="36" customHeight="1">
@@ -1540,7 +1540,7 @@
         <x:v>events/travel_events/travel_danger_events_oltner.txt:801</x:v>
       </x:c>
       <x:c r="G50" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6262</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6261</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="36" customHeight="1">
@@ -1563,7 +1563,7 @@
         <x:v>events/travel_events/travel_danger_events_dan.txt:131</x:v>
       </x:c>
       <x:c r="G51" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1019</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1018</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="36" customHeight="1">
@@ -1586,7 +1586,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:1274</x:v>
       </x:c>
       <x:c r="G52" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:393</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:392</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="36" customHeight="1">
@@ -1609,7 +1609,7 @@
         <x:v>events/travel_events/travel_events_filippa.txt:3784</x:v>
       </x:c>
       <x:c r="G53" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6381</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6380</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="36" customHeight="1">
@@ -1632,7 +1632,7 @@
         <x:v>events/activities/hunt_activity/hunt_events.txt:16889</x:v>
       </x:c>
       <x:c r="G54" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:632</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:631</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="36" customHeight="1">
@@ -1678,7 +1678,7 @@
         <x:v>events/activities/feast_activity/murder_feast_events.txt:748</x:v>
       </x:c>
       <x:c r="G56" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12308</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12307</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="36" customHeight="1">
@@ -1701,7 +1701,7 @@
         <x:v>events/stress_events/stress_threshold_events.txt:9820</x:v>
       </x:c>
       <x:c r="G57" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:1287</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:1286</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="36" customHeight="1">
@@ -1724,7 +1724,7 @@
         <x:v>events/activities/funeral_activity/funeral_events.txt:2070</x:v>
       </x:c>
       <x:c r="G58" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:13022</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:13021</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="36" customHeight="1">
@@ -1770,7 +1770,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:11554</x:v>
       </x:c>
       <x:c r="G60" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11540</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11539</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="36" customHeight="1">
@@ -1793,7 +1793,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:7415</x:v>
       </x:c>
       <x:c r="G61" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11463</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11462</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="36" customHeight="1">
@@ -1816,7 +1816,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:3438</x:v>
       </x:c>
       <x:c r="G62" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11368</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11367</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="36" customHeight="1">
@@ -1839,7 +1839,7 @@
         <x:v>events/activities/hunt_activity/hunt_events.txt:14343</x:v>
       </x:c>
       <x:c r="G63" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:132</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:131</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="36" customHeight="1">
@@ -1908,7 +1908,7 @@
         <x:v>events/activities/hunt_activity/jb_hunt_events.txt:3447</x:v>
       </x:c>
       <x:c r="G66" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10370</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10369</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="36" customHeight="1">
@@ -1954,7 +1954,7 @@
         <x:v>events/board_game_events.txt:122</x:v>
       </x:c>
       <x:c r="G68" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:273</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:272</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="36" customHeight="1">
@@ -1977,7 +1977,7 @@
         <x:v>events/activities/hunt_activity/jb_hunt_events.txt:794</x:v>
       </x:c>
       <x:c r="G69" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9816</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9815</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="36" customHeight="1">
@@ -2000,7 +2000,7 @@
         <x:v>events/activities/hunt_activity/hunt_events_anna.txt:315</x:v>
       </x:c>
       <x:c r="G70" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9957</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9956</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="36" customHeight="1">
@@ -2092,7 +2092,7 @@
         <x:v>events/health_events.txt:9266</x:v>
       </x:c>
       <x:c r="G74" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_health_options.txt:25</x:v>
+        <x:v>AuraClash/events/ac_vanilla_health_options.txt:24</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="36" customHeight="1">
@@ -2115,7 +2115,7 @@
         <x:v>events/health_events.txt:9639</x:v>
       </x:c>
       <x:c r="G75" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_health_options.txt:458</x:v>
+        <x:v>AuraClash/events/ac_vanilla_health_options.txt:457</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="32" customHeight="1">
@@ -2138,7 +2138,7 @@
         <x:v>events/dlc/pam/pam_secular_faith_events.txt:3398</x:v>
       </x:c>
       <x:c r="G76" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:835</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:834</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="32" customHeight="1">
@@ -2184,7 +2184,7 @@
         <x:v>events/dlc/ach/ach_coronation_events.txt:3409</x:v>
       </x:c>
       <x:c r="G78" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:108</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:107</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="32" customHeight="1">
@@ -2460,7 +2460,7 @@
         <x:v>events/dlc/ce1/epidemic_events.txt:2097</x:v>
       </x:c>
       <x:c r="G90" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:1098</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:1097</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="32" customHeight="1">
@@ -2713,7 +2713,7 @@
         <x:v>events/activities/hold_court_activity/hold_court_events_general.txt:4849</x:v>
       </x:c>
       <x:c r="G101" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1578</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1577</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="36" customHeight="1">
@@ -2759,7 +2759,7 @@
         <x:v>events/activities/hold_court_activity/hold_court_events_general.txt:5514</x:v>
       </x:c>
       <x:c r="G103" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1238</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1237</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="32" customHeight="1">
@@ -2828,7 +2828,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="G106" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="32" customHeight="1">
@@ -2851,7 +2851,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:3953</x:v>
       </x:c>
       <x:c r="G107" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4119</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4118</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="32" customHeight="1">
@@ -2874,7 +2874,7 @@
         <x:v>events/activities/tournaments/tournament_events.txt:12399</x:v>
       </x:c>
       <x:c r="G108" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10642</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10641</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="36" customHeight="1">
@@ -2897,7 +2897,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:1629</x:v>
       </x:c>
       <x:c r="G109" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5088</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5087</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="36" customHeight="1">
@@ -2920,7 +2920,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:1330</x:v>
       </x:c>
       <x:c r="G110" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4765</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4764</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="32" customHeight="1">
@@ -2943,7 +2943,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:7650</x:v>
       </x:c>
       <x:c r="G111" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6105</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6104</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="32" customHeight="1">
@@ -2966,7 +2966,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:10910</x:v>
       </x:c>
       <x:c r="G112" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6695</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6694</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="36" customHeight="1">
@@ -2989,7 +2989,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:11182</x:v>
       </x:c>
       <x:c r="G113" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5460</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5459</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="32" customHeight="1">
@@ -3012,7 +3012,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:11392</x:v>
       </x:c>
       <x:c r="G114" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5694</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5693</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="32" customHeight="1">
@@ -3035,7 +3035,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:12024</x:v>
       </x:c>
       <x:c r="G115" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5883</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5882</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="32" customHeight="1">
@@ -3058,7 +3058,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6464</x:v>
       </x:c>
       <x:c r="G116" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2431</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2430</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="32" customHeight="1">
@@ -3081,7 +3081,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:6444</x:v>
       </x:c>
       <x:c r="G117" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4444</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4443</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="32" customHeight="1">
@@ -3104,7 +3104,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:2995</x:v>
       </x:c>
       <x:c r="G118" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3919</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3918</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="32" customHeight="1">
@@ -3127,7 +3127,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:885</x:v>
       </x:c>
       <x:c r="G119" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8478</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8477</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="32" customHeight="1">
@@ -3150,7 +3150,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:5953</x:v>
       </x:c>
       <x:c r="G120" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3114</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3113</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="32" customHeight="1">
@@ -3173,7 +3173,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:1893</x:v>
       </x:c>
       <x:c r="G121" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2932</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2931</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="32" customHeight="1">
@@ -3242,7 +3242,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6118</x:v>
       </x:c>
       <x:c r="G124" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3315</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3314</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="32" customHeight="1">
@@ -3265,7 +3265,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6295</x:v>
       </x:c>
       <x:c r="G125" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3528</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3527</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="32" customHeight="1">
@@ -3288,7 +3288,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:12820</x:v>
       </x:c>
       <x:c r="G126" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7997</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7996</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="32" customHeight="1">
@@ -3311,7 +3311,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:12366</x:v>
       </x:c>
       <x:c r="G127" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7733</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7732</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="32" customHeight="1">
@@ -3357,7 +3357,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:11800</x:v>
       </x:c>
       <x:c r="G129" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9627</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9626</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="32" customHeight="1">
@@ -3380,7 +3380,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13075</x:v>
       </x:c>
       <x:c r="G130" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8276</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8275</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="32" customHeight="1">
@@ -3403,7 +3403,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:3158</x:v>
       </x:c>
       <x:c r="G131" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3744</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3743</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="32" customHeight="1">
@@ -3426,7 +3426,7 @@
         <x:v>events/activities/tournaments/jb_recital_contest_events.txt:767</x:v>
       </x:c>
       <x:c r="G132" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7594</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7593</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="32" customHeight="1">
@@ -3449,7 +3449,7 @@
         <x:v>events/activities/tournaments/jason_first_race_event.txt:21</x:v>
       </x:c>
       <x:c r="G133" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8997</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8996</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="32" customHeight="1">
@@ -3472,7 +3472,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:9726</x:v>
       </x:c>
       <x:c r="G134" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6842</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6841</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="32" customHeight="1">
@@ -3495,7 +3495,7 @@
         <x:v>events/activities/tournaments/jb_recital_contest_events.txt:10</x:v>
       </x:c>
       <x:c r="G135" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6965</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6964</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="32" customHeight="1">
@@ -3518,7 +3518,7 @@
         <x:v>events/activities/tournaments/jb_recital_contest_events.txt:643</x:v>
       </x:c>
       <x:c r="G136" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7447</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7446</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="32" customHeight="1">
@@ -3541,7 +3541,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:8925</x:v>
       </x:c>
       <x:c r="G137" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6255</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6254</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="32" customHeight="1">
@@ -3587,7 +3587,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:9174</x:v>
       </x:c>
       <x:c r="G139" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6539</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6538</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="32" customHeight="1">
@@ -3610,7 +3610,7 @@
         <x:v>events/activities/tour_activity/tour_phase_host_a_dinner.txt:4823</x:v>
       </x:c>
       <x:c r="G140" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_fatal_options.txt:209</x:v>
+        <x:v>AuraClash/events/ac_vanilla_fatal_options.txt:208</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="32" customHeight="1">
@@ -3633,7 +3633,7 @@
         <x:v>events/activities/tour_activity/tour_phase_tour_grounds.txt:2970</x:v>
       </x:c>
       <x:c r="G141" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12804</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12803</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="32" customHeight="1">
@@ -3656,7 +3656,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:13504</x:v>
       </x:c>
       <x:c r="G142" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2760</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2759</x:v>
       </x:c>
     </x:row>
     <x:row r="143" ht="32" customHeight="1">
@@ -3679,7 +3679,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:13350</x:v>
       </x:c>
       <x:c r="G143" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2594</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2593</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="36" customHeight="1">
@@ -3800,7 +3800,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54c7c8bdca6f41f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf027996c10f44af1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4195,7 +4195,7 @@
         <x:v>events/dlc/tgp/tgp_japan_yearly_events_ariana.txt:5213</x:v>
       </x:c>
       <x:c r="J14" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:3160</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:3159</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="50" customHeight="1">
@@ -4579,7 +4579,7 @@
         <x:v>events/dlc/tgp/tgp_governor_contract_events.txt:2872</x:v>
       </x:c>
       <x:c r="J26" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2326</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2325</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="36" customHeight="1">
@@ -4739,7 +4739,7 @@
         <x:v>events/dlc/tgp/tgp_natural_disaster_flavor_events.txt:585</x:v>
       </x:c>
       <x:c r="J31" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2497</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2496</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="50" customHeight="1">
@@ -4963,7 +4963,7 @@
         <x:v>events/dlc/tgp/tgp_natural_disaster_flavor_events.txt:259</x:v>
       </x:c>
       <x:c r="J38" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2836</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2835</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="50" customHeight="1">
@@ -4995,7 +4995,7 @@
         <x:v>events/dlc/tgp/tgp_natural_disaster_flavor_events.txt:259</x:v>
       </x:c>
       <x:c r="J39" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2836</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:2835</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="36" customHeight="1">
@@ -5155,7 +5155,7 @@
         <x:v>events/travel_events/travel_danger_events_arky.txt:143</x:v>
       </x:c>
       <x:c r="J44" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4399</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4398</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="36" customHeight="1">
@@ -5187,7 +5187,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:529</x:v>
       </x:c>
       <x:c r="J45" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10960</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10959</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="36" customHeight="1">
@@ -5219,7 +5219,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:529</x:v>
       </x:c>
       <x:c r="J46" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10960</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10959</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="36" customHeight="1">
@@ -5251,7 +5251,7 @@
         <x:v>events/health_events.txt:9507</x:v>
       </x:c>
       <x:c r="J47" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_health_options.txt:295</x:v>
+        <x:v>AuraClash/events/ac_vanilla_health_options.txt:294</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="36" customHeight="1">
@@ -5283,7 +5283,7 @@
         <x:v>events/health_events.txt:9507</x:v>
       </x:c>
       <x:c r="J48" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_health_options.txt:295</x:v>
+        <x:v>AuraClash/events/ac_vanilla_health_options.txt:294</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="36" customHeight="1">
@@ -5347,7 +5347,7 @@
         <x:v>events/activities/hunt_activity/hunt_events_anna.txt:437</x:v>
       </x:c>
       <x:c r="J50" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10137</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10136</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="36" customHeight="1">
@@ -5379,7 +5379,7 @@
         <x:v>events/activities/feast_activity/main_events/feast_default_events.txt:12335</x:v>
       </x:c>
       <x:c r="J51" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11810</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11809</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="36" customHeight="1">
@@ -5411,7 +5411,7 @@
         <x:v>events/travel_events/travel_events.txt:880</x:v>
       </x:c>
       <x:c r="J52" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4201</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4200</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="36" customHeight="1">
@@ -5443,7 +5443,7 @@
         <x:v>events/travel_events/travel_danger_events_joe.txt:135</x:v>
       </x:c>
       <x:c r="J53" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6015</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6014</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="36" customHeight="1">
@@ -5475,7 +5475,7 @@
         <x:v>events/travel_events/travel_danger_events_joe.txt:135</x:v>
       </x:c>
       <x:c r="J54" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6015</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6014</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="36" customHeight="1">
@@ -5507,7 +5507,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:1466</x:v>
       </x:c>
       <x:c r="J55" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1318</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1317</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="50" customHeight="1">
@@ -5539,7 +5539,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:582</x:v>
       </x:c>
       <x:c r="J56" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1883</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1882</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="36" customHeight="1">
@@ -5571,7 +5571,7 @@
         <x:v>events/travel_events/travel_events_veronica.txt:3064</x:v>
       </x:c>
       <x:c r="J57" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3006</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3005</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="36" customHeight="1">
@@ -5603,7 +5603,7 @@
         <x:v>events/travel_events/travel_events_veronica.txt:3064</x:v>
       </x:c>
       <x:c r="J58" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3006</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3005</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="36" customHeight="1">
@@ -5635,7 +5635,7 @@
         <x:v>events/travel_events/travel_events_veronica.txt:3064</x:v>
       </x:c>
       <x:c r="J59" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3006</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3005</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="36" customHeight="1">
@@ -5667,7 +5667,7 @@
         <x:v>events/travel_events/travel_events_veronica.txt:3064</x:v>
       </x:c>
       <x:c r="J60" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3006</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3005</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="50" customHeight="1">
@@ -5699,7 +5699,7 @@
         <x:v>events/travel_events/travel_danger_events_joe.txt:2211</x:v>
       </x:c>
       <x:c r="J61" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_fatal_options.txt:17</x:v>
+        <x:v>AuraClash/events/ac_vanilla_fatal_options.txt:16</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="36" customHeight="1">
@@ -5731,7 +5731,7 @@
         <x:v>events/travel_events/travel_danger_events.txt:613</x:v>
       </x:c>
       <x:c r="J62" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:2214</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:2213</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="50" customHeight="1">
@@ -5763,7 +5763,7 @@
         <x:v>events/travel_events/travel_events_veronica.txt:4531</x:v>
       </x:c>
       <x:c r="J63" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:7107</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:7106</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="36" customHeight="1">
@@ -5795,7 +5795,7 @@
         <x:v>events/travel_events/travel_events_veronica.txt:4531</x:v>
       </x:c>
       <x:c r="J64" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:7107</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:7106</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="36" customHeight="1">
@@ -5827,7 +5827,7 @@
         <x:v>events/travel_events/travel_events_veronica.txt:4531</x:v>
       </x:c>
       <x:c r="J65" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:7107</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:7106</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="36" customHeight="1">
@@ -5859,7 +5859,7 @@
         <x:v>events/travel_events/travel_danger_events_joe.txt:2364</x:v>
       </x:c>
       <x:c r="J66" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3334</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3333</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="36" customHeight="1">
@@ -5891,7 +5891,7 @@
         <x:v>events/travel_events/travel_danger_events_joe.txt:2364</x:v>
       </x:c>
       <x:c r="J67" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3334</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:3333</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="36" customHeight="1">
@@ -5923,7 +5923,7 @@
         <x:v>events/travel_events/travel_danger_events.txt:806</x:v>
       </x:c>
       <x:c r="J68" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1132</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1131</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="36" customHeight="1">
@@ -5955,7 +5955,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:9</x:v>
       </x:c>
       <x:c r="J69" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:2420</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:2419</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="36" customHeight="1">
@@ -5987,7 +5987,7 @@
         <x:v>events/travel_events/travel_danger_events_filippa.txt:8</x:v>
       </x:c>
       <x:c r="J70" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:608</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:607</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="36" customHeight="1">
@@ -6019,7 +6019,7 @@
         <x:v>events/travel_events/travel_danger_events_oltner.txt:922</x:v>
       </x:c>
       <x:c r="J71" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4039</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:4038</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="36" customHeight="1">
@@ -6051,7 +6051,7 @@
         <x:v>events/travel_events/travel_danger_events_ariana.txt:92</x:v>
       </x:c>
       <x:c r="J72" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:5058</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:5057</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="36" customHeight="1">
@@ -6083,7 +6083,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:949</x:v>
       </x:c>
       <x:c r="J73" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1544</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1543</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="36" customHeight="1">
@@ -6115,7 +6115,7 @@
         <x:v>events/travel_events/travel_danger_events_oltner.txt:301</x:v>
       </x:c>
       <x:c r="J74" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:3005</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:3004</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="36" customHeight="1">
@@ -6147,7 +6147,7 @@
         <x:v>events/travel_events/travel_danger_events_oltner.txt:801</x:v>
       </x:c>
       <x:c r="J75" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6262</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6261</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="36" customHeight="1">
@@ -6179,7 +6179,7 @@
         <x:v>events/travel_events/travel_danger_events_dan.txt:131</x:v>
       </x:c>
       <x:c r="J76" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1019</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:1018</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="36" customHeight="1">
@@ -6211,7 +6211,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:1274</x:v>
       </x:c>
       <x:c r="J77" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:393</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:392</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="36" customHeight="1">
@@ -6243,7 +6243,7 @@
         <x:v>events/travel_events/travel_danger_events_klank.txt:1274</x:v>
       </x:c>
       <x:c r="J78" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:393</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:392</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="36" customHeight="1">
@@ -6275,7 +6275,7 @@
         <x:v>events/travel_events/travel_events_filippa.txt:3784</x:v>
       </x:c>
       <x:c r="J79" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6381</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6380</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="50" customHeight="1">
@@ -6307,7 +6307,7 @@
         <x:v>events/travel_events/travel_events_filippa.txt:3784</x:v>
       </x:c>
       <x:c r="J80" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6381</x:v>
+        <x:v>AuraClash/events/ac_vanilla_travel_options.txt:6380</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="36" customHeight="1">
@@ -6339,7 +6339,7 @@
         <x:v>events/activities/hunt_activity/hunt_events.txt:16889</x:v>
       </x:c>
       <x:c r="J81" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:632</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:631</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="36" customHeight="1">
@@ -6371,7 +6371,7 @@
         <x:v>events/activities/hunt_activity/hunt_events.txt:16889</x:v>
       </x:c>
       <x:c r="J82" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:632</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:631</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="36" customHeight="1">
@@ -6435,7 +6435,7 @@
         <x:v>events/activities/feast_activity/murder_feast_events.txt:748</x:v>
       </x:c>
       <x:c r="J84" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12308</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12307</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="50" customHeight="1">
@@ -6467,7 +6467,7 @@
         <x:v>events/activities/feast_activity/murder_feast_events.txt:748</x:v>
       </x:c>
       <x:c r="J85" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12308</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12307</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="50" customHeight="1">
@@ -6499,7 +6499,7 @@
         <x:v>events/activities/feast_activity/murder_feast_events.txt:748</x:v>
       </x:c>
       <x:c r="J86" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12308</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12307</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="36" customHeight="1">
@@ -6531,7 +6531,7 @@
         <x:v>events/stress_events/stress_threshold_events.txt:9820</x:v>
       </x:c>
       <x:c r="J87" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:1287</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:1286</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="36" customHeight="1">
@@ -6563,7 +6563,7 @@
         <x:v>events/activities/funeral_activity/funeral_events.txt:2070</x:v>
       </x:c>
       <x:c r="J88" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:13022</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:13021</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="36" customHeight="1">
@@ -6659,7 +6659,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:11554</x:v>
       </x:c>
       <x:c r="J91" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11540</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11539</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="36" customHeight="1">
@@ -6691,7 +6691,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:11554</x:v>
       </x:c>
       <x:c r="J92" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11540</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11539</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="36" customHeight="1">
@@ -6723,7 +6723,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:7415</x:v>
       </x:c>
       <x:c r="J93" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11463</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11462</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="36" customHeight="1">
@@ -6755,7 +6755,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:7415</x:v>
       </x:c>
       <x:c r="J94" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11463</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11462</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="36" customHeight="1">
@@ -6787,7 +6787,7 @@
         <x:v>events/activities/pilgrimage_activity/pilgrimage_events.txt:3438</x:v>
       </x:c>
       <x:c r="J95" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11368</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:11367</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="36" customHeight="1">
@@ -6819,7 +6819,7 @@
         <x:v>events/activities/hunt_activity/hunt_events.txt:14343</x:v>
       </x:c>
       <x:c r="J96" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:132</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:131</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="36" customHeight="1">
@@ -6979,7 +6979,7 @@
         <x:v>events/activities/hunt_activity/jb_hunt_events.txt:3447</x:v>
       </x:c>
       <x:c r="J101" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10370</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10369</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="36" customHeight="1">
@@ -7011,7 +7011,7 @@
         <x:v>events/activities/hunt_activity/jb_hunt_events.txt:3447</x:v>
       </x:c>
       <x:c r="J102" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10370</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10369</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="36" customHeight="1">
@@ -7139,7 +7139,7 @@
         <x:v>events/board_game_events.txt:122</x:v>
       </x:c>
       <x:c r="J106" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:273</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:272</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="36" customHeight="1">
@@ -7171,7 +7171,7 @@
         <x:v>events/activities/hunt_activity/jb_hunt_events.txt:794</x:v>
       </x:c>
       <x:c r="J107" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9816</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9815</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="36" customHeight="1">
@@ -7203,7 +7203,7 @@
         <x:v>events/activities/hunt_activity/hunt_events_anna.txt:315</x:v>
       </x:c>
       <x:c r="J108" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9957</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9956</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="36" customHeight="1">
@@ -7235,7 +7235,7 @@
         <x:v>events/activities/hunt_activity/hunt_events_anna.txt:315</x:v>
       </x:c>
       <x:c r="J109" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9957</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9956</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="36" customHeight="1">
@@ -7267,7 +7267,7 @@
         <x:v>events/activities/hunt_activity/hunt_events_anna.txt:315</x:v>
       </x:c>
       <x:c r="J110" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9957</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9956</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="50" customHeight="1">
@@ -7555,7 +7555,7 @@
         <x:v>events/health_events.txt:9266</x:v>
       </x:c>
       <x:c r="J119" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_health_options.txt:25</x:v>
+        <x:v>AuraClash/events/ac_vanilla_health_options.txt:24</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="36" customHeight="1">
@@ -7587,7 +7587,7 @@
         <x:v>events/health_events.txt:9266</x:v>
       </x:c>
       <x:c r="J120" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_health_options.txt:25</x:v>
+        <x:v>AuraClash/events/ac_vanilla_health_options.txt:24</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="36" customHeight="1">
@@ -7619,7 +7619,7 @@
         <x:v>events/health_events.txt:9639</x:v>
       </x:c>
       <x:c r="J121" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_health_options.txt:458</x:v>
+        <x:v>AuraClash/events/ac_vanilla_health_options.txt:457</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="36" customHeight="1">
@@ -7651,7 +7651,7 @@
         <x:v>events/health_events.txt:9639</x:v>
       </x:c>
       <x:c r="J122" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_health_options.txt:458</x:v>
+        <x:v>AuraClash/events/ac_vanilla_health_options.txt:457</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="36" customHeight="1">
@@ -7683,7 +7683,7 @@
         <x:v>events/dlc/pam/pam_secular_faith_events.txt:3398</x:v>
       </x:c>
       <x:c r="J123" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:835</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:834</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="36" customHeight="1">
@@ -7747,7 +7747,7 @@
         <x:v>events/dlc/ach/ach_coronation_events.txt:3409</x:v>
       </x:c>
       <x:c r="J125" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:108</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:107</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="50" customHeight="1">
@@ -8419,7 +8419,7 @@
         <x:v>events/dlc/ce1/epidemic_events.txt:2097</x:v>
       </x:c>
       <x:c r="J146" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_school_options.txt:1098</x:v>
+        <x:v>AuraClash/events/ac_vanilla_school_options.txt:1097</x:v>
       </x:c>
     </x:row>
     <x:row r="147" ht="36" customHeight="1">
@@ -9315,7 +9315,7 @@
         <x:v>events/activities/hold_court_activity/hold_court_events_general.txt:4849</x:v>
       </x:c>
       <x:c r="J174" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1578</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1577</x:v>
       </x:c>
     </x:row>
     <x:row r="175" ht="36" customHeight="1">
@@ -9347,7 +9347,7 @@
         <x:v>events/activities/hold_court_activity/hold_court_events_general.txt:4849</x:v>
       </x:c>
       <x:c r="J175" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1578</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1577</x:v>
       </x:c>
     </x:row>
     <x:row r="176" ht="36" customHeight="1">
@@ -9411,7 +9411,7 @@
         <x:v>events/activities/hold_court_activity/hold_court_events_general.txt:5514</x:v>
       </x:c>
       <x:c r="J177" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1238</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activity_options.txt:1237</x:v>
       </x:c>
     </x:row>
     <x:row r="178" ht="36" customHeight="1">
@@ -9571,7 +9571,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="J182" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="183" ht="50" customHeight="1">
@@ -9603,7 +9603,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="J183" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="50" customHeight="1">
@@ -9635,7 +9635,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="J184" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="185" ht="50" customHeight="1">
@@ -9667,7 +9667,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="J185" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="186" ht="50" customHeight="1">
@@ -9699,7 +9699,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="J186" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="187" ht="50" customHeight="1">
@@ -9731,7 +9731,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="J187" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="188" ht="50" customHeight="1">
@@ -9763,7 +9763,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="J188" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="189" ht="50" customHeight="1">
@@ -9795,7 +9795,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="J189" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="190" ht="50" customHeight="1">
@@ -9827,7 +9827,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13777</x:v>
       </x:c>
       <x:c r="J190" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8656</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8655</x:v>
       </x:c>
     </x:row>
     <x:row r="191" ht="36" customHeight="1">
@@ -9859,7 +9859,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:3953</x:v>
       </x:c>
       <x:c r="J191" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4119</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4118</x:v>
       </x:c>
     </x:row>
     <x:row r="192" ht="36" customHeight="1">
@@ -9891,7 +9891,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:3953</x:v>
       </x:c>
       <x:c r="J192" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4119</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4118</x:v>
       </x:c>
     </x:row>
     <x:row r="193" ht="36" customHeight="1">
@@ -9923,7 +9923,7 @@
         <x:v>events/activities/tournaments/tournament_events.txt:12399</x:v>
       </x:c>
       <x:c r="J193" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10642</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10641</x:v>
       </x:c>
     </x:row>
     <x:row r="194" ht="36" customHeight="1">
@@ -9955,7 +9955,7 @@
         <x:v>events/activities/tournaments/tournament_events.txt:12399</x:v>
       </x:c>
       <x:c r="J194" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10642</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10641</x:v>
       </x:c>
     </x:row>
     <x:row r="195" ht="36" customHeight="1">
@@ -9987,7 +9987,7 @@
         <x:v>events/activities/tournaments/tournament_events.txt:12399</x:v>
       </x:c>
       <x:c r="J195" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10642</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:10641</x:v>
       </x:c>
     </x:row>
     <x:row r="196" ht="50" customHeight="1">
@@ -10019,7 +10019,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:1629</x:v>
       </x:c>
       <x:c r="J196" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5088</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5087</x:v>
       </x:c>
     </x:row>
     <x:row r="197" ht="50" customHeight="1">
@@ -10051,7 +10051,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:1629</x:v>
       </x:c>
       <x:c r="J197" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5088</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5087</x:v>
       </x:c>
     </x:row>
     <x:row r="198" ht="50" customHeight="1">
@@ -10083,7 +10083,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:1330</x:v>
       </x:c>
       <x:c r="J198" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4765</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4764</x:v>
       </x:c>
     </x:row>
     <x:row r="199" ht="50" customHeight="1">
@@ -10115,7 +10115,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:1330</x:v>
       </x:c>
       <x:c r="J199" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4765</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4764</x:v>
       </x:c>
     </x:row>
     <x:row r="200" ht="50" customHeight="1">
@@ -10147,7 +10147,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:7650</x:v>
       </x:c>
       <x:c r="J200" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6105</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6104</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="36" customHeight="1">
@@ -10179,7 +10179,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:10910</x:v>
       </x:c>
       <x:c r="J201" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6695</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6694</x:v>
       </x:c>
     </x:row>
     <x:row r="202" ht="50" customHeight="1">
@@ -10211,7 +10211,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:11182</x:v>
       </x:c>
       <x:c r="J202" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5460</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5459</x:v>
       </x:c>
     </x:row>
     <x:row r="203" ht="50" customHeight="1">
@@ -10243,7 +10243,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:11182</x:v>
       </x:c>
       <x:c r="J203" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5460</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5459</x:v>
       </x:c>
     </x:row>
     <x:row r="204" ht="50" customHeight="1">
@@ -10275,7 +10275,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:11392</x:v>
       </x:c>
       <x:c r="J204" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5694</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5693</x:v>
       </x:c>
     </x:row>
     <x:row r="205" ht="50" customHeight="1">
@@ -10307,7 +10307,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:11392</x:v>
       </x:c>
       <x:c r="J205" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5694</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5693</x:v>
       </x:c>
     </x:row>
     <x:row r="206" ht="50" customHeight="1">
@@ -10339,7 +10339,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:12024</x:v>
       </x:c>
       <x:c r="J206" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5883</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5882</x:v>
       </x:c>
     </x:row>
     <x:row r="207" ht="50" customHeight="1">
@@ -10371,7 +10371,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:12024</x:v>
       </x:c>
       <x:c r="J207" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5883</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:5882</x:v>
       </x:c>
     </x:row>
     <x:row r="208" ht="50" customHeight="1">
@@ -10403,7 +10403,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6464</x:v>
       </x:c>
       <x:c r="J208" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2431</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2430</x:v>
       </x:c>
     </x:row>
     <x:row r="209" ht="50" customHeight="1">
@@ -10435,7 +10435,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:6444</x:v>
       </x:c>
       <x:c r="J209" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4444</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4443</x:v>
       </x:c>
     </x:row>
     <x:row r="210" ht="50" customHeight="1">
@@ -10467,7 +10467,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:6444</x:v>
       </x:c>
       <x:c r="J210" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4444</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:4443</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="36" customHeight="1">
@@ -10499,7 +10499,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:2995</x:v>
       </x:c>
       <x:c r="J211" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3919</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3918</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="36" customHeight="1">
@@ -10531,7 +10531,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:2995</x:v>
       </x:c>
       <x:c r="J212" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3919</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3918</x:v>
       </x:c>
     </x:row>
     <x:row r="213" ht="50" customHeight="1">
@@ -10563,7 +10563,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:885</x:v>
       </x:c>
       <x:c r="J213" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8478</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8477</x:v>
       </x:c>
     </x:row>
     <x:row r="214" ht="50" customHeight="1">
@@ -10595,7 +10595,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:885</x:v>
       </x:c>
       <x:c r="J214" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8478</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8477</x:v>
       </x:c>
     </x:row>
     <x:row r="215" ht="50" customHeight="1">
@@ -10627,7 +10627,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:885</x:v>
       </x:c>
       <x:c r="J215" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8478</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8477</x:v>
       </x:c>
     </x:row>
     <x:row r="216" ht="50" customHeight="1">
@@ -10659,7 +10659,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:5953</x:v>
       </x:c>
       <x:c r="J216" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3114</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3113</x:v>
       </x:c>
     </x:row>
     <x:row r="217" ht="50" customHeight="1">
@@ -10691,7 +10691,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:5953</x:v>
       </x:c>
       <x:c r="J217" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3114</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3113</x:v>
       </x:c>
     </x:row>
     <x:row r="218" ht="50" customHeight="1">
@@ -10723,7 +10723,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:5953</x:v>
       </x:c>
       <x:c r="J218" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3114</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3113</x:v>
       </x:c>
     </x:row>
     <x:row r="219" ht="50" customHeight="1">
@@ -10755,7 +10755,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:1893</x:v>
       </x:c>
       <x:c r="J219" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2932</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2931</x:v>
       </x:c>
     </x:row>
     <x:row r="220" ht="50" customHeight="1">
@@ -10787,7 +10787,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:1893</x:v>
       </x:c>
       <x:c r="J220" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2932</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2931</x:v>
       </x:c>
     </x:row>
     <x:row r="221" ht="50" customHeight="1">
@@ -10819,7 +10819,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:1893</x:v>
       </x:c>
       <x:c r="J221" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2932</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2931</x:v>
       </x:c>
     </x:row>
     <x:row r="222" ht="36" customHeight="1">
@@ -10979,7 +10979,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6118</x:v>
       </x:c>
       <x:c r="J226" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3315</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3314</x:v>
       </x:c>
     </x:row>
     <x:row r="227" ht="50" customHeight="1">
@@ -11011,7 +11011,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6118</x:v>
       </x:c>
       <x:c r="J227" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3315</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3314</x:v>
       </x:c>
     </x:row>
     <x:row r="228" ht="50" customHeight="1">
@@ -11043,7 +11043,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6118</x:v>
       </x:c>
       <x:c r="J228" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3315</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3314</x:v>
       </x:c>
     </x:row>
     <x:row r="229" ht="50" customHeight="1">
@@ -11075,7 +11075,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6295</x:v>
       </x:c>
       <x:c r="J229" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3528</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3527</x:v>
       </x:c>
     </x:row>
     <x:row r="230" ht="50" customHeight="1">
@@ -11107,7 +11107,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6295</x:v>
       </x:c>
       <x:c r="J230" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3528</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3527</x:v>
       </x:c>
     </x:row>
     <x:row r="231" ht="50" customHeight="1">
@@ -11139,7 +11139,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6295</x:v>
       </x:c>
       <x:c r="J231" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3528</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3527</x:v>
       </x:c>
     </x:row>
     <x:row r="232" ht="50" customHeight="1">
@@ -11171,7 +11171,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:6295</x:v>
       </x:c>
       <x:c r="J232" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3528</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3527</x:v>
       </x:c>
     </x:row>
     <x:row r="233" ht="50" customHeight="1">
@@ -11203,7 +11203,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:12820</x:v>
       </x:c>
       <x:c r="J233" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7997</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7996</x:v>
       </x:c>
     </x:row>
     <x:row r="234" ht="50" customHeight="1">
@@ -11235,7 +11235,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:12820</x:v>
       </x:c>
       <x:c r="J234" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7997</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7996</x:v>
       </x:c>
     </x:row>
     <x:row r="235" ht="50" customHeight="1">
@@ -11267,7 +11267,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:12366</x:v>
       </x:c>
       <x:c r="J235" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7733</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7732</x:v>
       </x:c>
     </x:row>
     <x:row r="236" ht="50" customHeight="1">
@@ -11299,7 +11299,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:12366</x:v>
       </x:c>
       <x:c r="J236" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7733</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7732</x:v>
       </x:c>
     </x:row>
     <x:row r="237" ht="36" customHeight="1">
@@ -11363,7 +11363,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:11800</x:v>
       </x:c>
       <x:c r="J238" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9627</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9626</x:v>
       </x:c>
     </x:row>
     <x:row r="239" ht="36" customHeight="1">
@@ -11395,7 +11395,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:11800</x:v>
       </x:c>
       <x:c r="J239" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9627</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9626</x:v>
       </x:c>
     </x:row>
     <x:row r="240" ht="36" customHeight="1">
@@ -11427,7 +11427,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:11800</x:v>
       </x:c>
       <x:c r="J240" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9627</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:9626</x:v>
       </x:c>
     </x:row>
     <x:row r="241" ht="50" customHeight="1">
@@ -11459,7 +11459,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13075</x:v>
       </x:c>
       <x:c r="J241" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8276</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8275</x:v>
       </x:c>
     </x:row>
     <x:row r="242" ht="50" customHeight="1">
@@ -11491,7 +11491,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:13075</x:v>
       </x:c>
       <x:c r="J242" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8276</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8275</x:v>
       </x:c>
     </x:row>
     <x:row r="243" ht="50" customHeight="1">
@@ -11523,7 +11523,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:3158</x:v>
       </x:c>
       <x:c r="J243" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3744</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3743</x:v>
       </x:c>
     </x:row>
     <x:row r="244" ht="50" customHeight="1">
@@ -11555,7 +11555,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:3158</x:v>
       </x:c>
       <x:c r="J244" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3744</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3743</x:v>
       </x:c>
     </x:row>
     <x:row r="245" ht="50" customHeight="1">
@@ -11587,7 +11587,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:3158</x:v>
       </x:c>
       <x:c r="J245" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3744</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3743</x:v>
       </x:c>
     </x:row>
     <x:row r="246" ht="50" customHeight="1">
@@ -11619,7 +11619,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:3158</x:v>
       </x:c>
       <x:c r="J246" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3744</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:3743</x:v>
       </x:c>
     </x:row>
     <x:row r="247" ht="50" customHeight="1">
@@ -11651,7 +11651,7 @@
         <x:v>events/activities/tournaments/jb_recital_contest_events.txt:767</x:v>
       </x:c>
       <x:c r="J247" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7594</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7593</x:v>
       </x:c>
     </x:row>
     <x:row r="248" ht="50" customHeight="1">
@@ -11683,7 +11683,7 @@
         <x:v>events/activities/tournaments/jb_recital_contest_events.txt:767</x:v>
       </x:c>
       <x:c r="J248" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7594</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7593</x:v>
       </x:c>
     </x:row>
     <x:row r="249" ht="36" customHeight="1">
@@ -11715,7 +11715,7 @@
         <x:v>events/activities/tournaments/jason_first_race_event.txt:21</x:v>
       </x:c>
       <x:c r="J249" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8997</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8996</x:v>
       </x:c>
     </x:row>
     <x:row r="250" ht="36" customHeight="1">
@@ -11747,7 +11747,7 @@
         <x:v>events/activities/tournaments/jason_first_race_event.txt:21</x:v>
       </x:c>
       <x:c r="J250" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8997</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8996</x:v>
       </x:c>
     </x:row>
     <x:row r="251" ht="36" customHeight="1">
@@ -11779,7 +11779,7 @@
         <x:v>events/activities/tournaments/jason_first_race_event.txt:21</x:v>
       </x:c>
       <x:c r="J251" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8997</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:8996</x:v>
       </x:c>
     </x:row>
     <x:row r="252" ht="50" customHeight="1">
@@ -11811,7 +11811,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:9726</x:v>
       </x:c>
       <x:c r="J252" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6842</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6841</x:v>
       </x:c>
     </x:row>
     <x:row r="253" ht="50" customHeight="1">
@@ -11843,7 +11843,7 @@
         <x:v>events/activities/tournaments/jb_recital_contest_events.txt:10</x:v>
       </x:c>
       <x:c r="J253" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6965</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6964</x:v>
       </x:c>
     </x:row>
     <x:row r="254" ht="50" customHeight="1">
@@ -11875,7 +11875,7 @@
         <x:v>events/activities/tournaments/jb_recital_contest_events.txt:10</x:v>
       </x:c>
       <x:c r="J254" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6965</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6964</x:v>
       </x:c>
     </x:row>
     <x:row r="255" ht="50" customHeight="1">
@@ -11907,7 +11907,7 @@
         <x:v>events/activities/tournaments/jb_recital_contest_events.txt:643</x:v>
       </x:c>
       <x:c r="J255" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7447</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7446</x:v>
       </x:c>
     </x:row>
     <x:row r="256" ht="50" customHeight="1">
@@ -11939,7 +11939,7 @@
         <x:v>events/activities/tournaments/jb_recital_contest_events.txt:643</x:v>
       </x:c>
       <x:c r="J256" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7447</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:7446</x:v>
       </x:c>
     </x:row>
     <x:row r="257" ht="50" customHeight="1">
@@ -11971,7 +11971,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:8925</x:v>
       </x:c>
       <x:c r="J257" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6255</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6254</x:v>
       </x:c>
     </x:row>
     <x:row r="258" ht="50" customHeight="1">
@@ -12003,7 +12003,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:8925</x:v>
       </x:c>
       <x:c r="J258" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6255</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6254</x:v>
       </x:c>
     </x:row>
     <x:row r="259" ht="50" customHeight="1">
@@ -12035,7 +12035,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:8925</x:v>
       </x:c>
       <x:c r="J259" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6255</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6254</x:v>
       </x:c>
     </x:row>
     <x:row r="260" ht="50" customHeight="1">
@@ -12067,7 +12067,7 @@
         <x:v>events/dlc/ep2/ep2_tournament_events.txt:9174</x:v>
       </x:c>
       <x:c r="J260" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6539</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:6538</x:v>
       </x:c>
     </x:row>
     <x:row r="261" ht="50" customHeight="1">
@@ -12099,7 +12099,7 @@
         <x:v>events/activities/tour_activity/tour_phase_host_a_dinner.txt:4823</x:v>
       </x:c>
       <x:c r="J261" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_fatal_options.txt:209</x:v>
+        <x:v>AuraClash/events/ac_vanilla_fatal_options.txt:208</x:v>
       </x:c>
     </x:row>
     <x:row r="262" ht="36" customHeight="1">
@@ -12131,7 +12131,7 @@
         <x:v>events/activities/tour_activity/tour_phase_tour_grounds.txt:2970</x:v>
       </x:c>
       <x:c r="J262" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12804</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12803</x:v>
       </x:c>
     </x:row>
     <x:row r="263" ht="36" customHeight="1">
@@ -12163,7 +12163,7 @@
         <x:v>events/activities/tour_activity/tour_phase_tour_grounds.txt:2970</x:v>
       </x:c>
       <x:c r="J263" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12804</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:12803</x:v>
       </x:c>
     </x:row>
     <x:row r="264" ht="50" customHeight="1">
@@ -12195,7 +12195,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:13504</x:v>
       </x:c>
       <x:c r="J264" s="20" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2760</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2759</x:v>
       </x:c>
     </x:row>
     <x:row r="265" ht="50" customHeight="1">
@@ -12227,7 +12227,7 @@
         <x:v>events/activities/tournaments/contest_events.txt:13350</x:v>
       </x:c>
       <x:c r="J265" s="21" t="str">
-        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2594</x:v>
+        <x:v>AuraClash/events/ac_vanilla_activities_options.txt:2593</x:v>
       </x:c>
     </x:row>
     <x:row r="266" ht="36" customHeight="1">
@@ -12521,7 +12521,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ac66d14ae214514"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf39aeea28ecc4c48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>